<commit_message>
Loop zonder errors, maar niet alle data aanwezig. Alles vanaf diagnostics uitgezet. WIP
</commit_message>
<xml_diff>
--- a/Input/Dataframes/nutri_markers.xlsx
+++ b/Input/Dataframes/nutri_markers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Werk\NifGo\Input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Werk\NifGo\Input\Dataframes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A002C46-2522-4356-8CAE-9AB502620449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36B482FA-2031-4407-BDDF-37F6F378A158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25800" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Export Nutri Markers 2202" sheetId="1" r:id="rId1"/>

</xml_diff>